<commit_message>
completato tripadvisor; sistemato alcune cose in generale
</commit_message>
<xml_diff>
--- a/datasets/general_data_dataset_tripadvisor.xlsx
+++ b/datasets/general_data_dataset_tripadvisor.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,6 +446,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>facilities</t>
         </is>
       </c>
@@ -471,6 +476,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>191 €</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Piscina, Lezioni di yoga, Bar/lounge, Spiaggia, Tiro con l'arco, Parco giochi per bambini, Area giochi interna per bambini, Parcheggio custodito, Teli da piscina/mare, Piscina all'aperto, Corsi di fitness, Ristorante, Colazione a buffet, Drink di benvenuto omaggio, Noleggio di biciclette, Canoismo, Campo da tennis, Noleggi di attrezzature per sport acquatici, Windsurf, Tour in bicicletta, Personale di intrattenimento, Intrattenimento serale, Karaoke, Ping pong, Attività per bambini/famiglie, Miniclub, Piscina per bambini, Giochi all'aperto per bambini, Seggioloni disponibili, Animali domestici ammessi, Servizio taxi, Sicurezza 24 ore su 24, Minimarket, Zanzariera, Lettini/sedie sdraio, Ombrelloni, Cassetta di pronto soccorso, Infermeria, Lavanderia self-service, Lavatrice, Camere insonorizzate, Aria condizionata, Spiaggia privata, Servizio di pulizia, Angolo cottura, TV a schermo piatto, Divano letto, Bidet, Cassaforte, Zona soggiorno, Divano, Armadio/cabina, Forno, Frigorifero, Piano cottura, Utensili da cucina, Cabina doccia, Asciugacapelli, Camere non fumatori, Camere per famiglie, </t>
         </is>
       </c>
@@ -496,6 +506,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>275 €</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Bar/lounge, Spiaggia, Tiro con l'arco, Parco giochi per bambini, Area giochi interna per bambini, Wi-Fi, Giochi da piscina, Piscina all'aperto, Piscina con estremità bassa, Ristorante, Colazione disponibile, Pasti per bambini, Menù dietetici speciali, Bar in piscina, Noleggio di biciclette, Canoismo, Escursioni, Campo da tennis, Parco acquatico, Windsurf, Aerobica, Personale di intrattenimento, Intrattenimento serale, Ping pong, Scivolo acquatico, Attività per bambini/famiglie, Miniclub, Piscina per bambini, Giochi all'aperto per bambini, Seggioloni disponibili, Passeggini, Animali domestici ammessi, Area barbecue, Minimarket, Negozio di articoli da regalo, Quotidiano, Negozi, Lettini/sedie sdraio, Ombrelloni, Bancomat in loco, Infermeria, Lavanderia self-service, Aria condizionata, Spiaggia privata, Servizio di pulizia, Cassaforte, Angolo cottura, Frigorifero, TV a schermo piatto, Bagno/doccia, Zona soggiorno, Piano cottura, Utensili da cucina, Camere per famiglie, </t>
         </is>
       </c>
@@ -521,6 +536,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>34 €</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Bar/lounge, Spiaggia, Campo da tennis, Attività per bambini/famiglie, Miniclub, Wi-Fi, Piscina all'aperto, Ristorante, Bar in piscina, Bar a bordo piscina, Personale di intrattenimento, Intrattenimento serale, Ping pong, Giochi all'aperto per bambini, Animali domestici ammessi, Minimarket, Lavanderia self-service, Aria condizionata, Spiaggia privata, Angolo cottura, Frigorifero, Utensili da cucina, TV a schermo piatto, Vista sull'oceano, </t>
         </is>
       </c>
@@ -546,6 +566,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>154 €</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Wi-Fi, Piscina, Bar/lounge, Noleggio di biciclette, Canoismo, Attività per bambini/famiglie, Miniclub, Piscina all'aperto, Piscina con estremità bassa, Piscina recintata, Ristorante, Snack bar, Campo da tennis, Ping pong, Piscina per bambini, Giochi all'aperto per bambini, Animali domestici ammessi, Navetta o servizio taxi gratis, Area barbecue, Lounge/sala TV in comune, Terrazza solarium, Servizio lavanderia, Lavanderia self-service, Spiaggia privata, Angolo cottura, Frigorifero, TV a schermo piatto, Camere per famiglie, </t>
         </is>
       </c>
@@ -571,6 +596,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Ristorante, Spiaggia, Noleggio di biciclette, Parco giochi per bambini, Area giochi interna per bambini, Parcheggio custodito, Wi-Fi, Vasca idromassaggio, Piscina all'aperto, Piscina con estremità bassa, Piscina recintata, Zona pranzo all'aperto, Snack bar, Aerobica, Freccette, Personale di intrattenimento, Intrattenimento serale, Ping pong, Attività per bambini/famiglie, Miniclub, Giochi all'aperto per bambini, Area barbecue, Minimarket, Hotel per non fumatori, Lounge/sala TV in comune, Lettini/sedie sdraio, Ombrelloni, Asciugatrice, Aria condizionata, Zona soggiorno, Divano, Appendiabiti, Bollitore per tè/caffè, Angolo cottura, TV a schermo piatto, Bidet, Bagni privati, Frigorifero, Piano cottura, Utensili da cucina, Cabina doccia, Camere non fumatori, Camere per famiglie, </t>
         </is>
       </c>
@@ -591,10 +621,15 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ho trascorso 3 giorni in questa struttura in un villino in muratura. Ho trovato un ambiente pulito, personale gentilissimo e disponibile verso ogni richiesta. Bella piscina .in mezza pensio ne ho trovato cibo curato e con buona scelta.  La spiaggia è raggiungibile con una bella passeggiata, ma se non si vuole passeggiare la struttura offre una navetta. Lo stabilimento balneare convenzionato con la struttura è ottimo. Biciclette disponibili per percorrere una bella ciclabile sul mare,ideale anche per piacevoli passeggiate.</t>
+          <t>Ci siamo innamorati di questa struttura un anno fa, quando l'abbiamo scoperta per puro caso; e quest'anno, al momento di prenotare le vacanze, non abbiamo avuto dubbi: Garden River di nuovo. Per chi come noi ha un budget limitato e cerca una struttura comoda e ben organizzata, le casette in muratura sono a nostro avviso la scelta ideale. Ovvio che, trovandosi in un camping immerso nel verde (e nel profumo) dei tigli, non bisogna scandalizzarsi se di tanto in tanto la formica, l'insettino, il geco si affacciano nelle casette... ma le costruzioni sono pulite, essenziali nel loro arredo, comode, fresche e, cosa essenziale per una famiglia di cinque persone come la nostra, comodissime da pulire. Specialmente il bagno, con la doccia che prende l'intera parete e consente di entrare in due (lo scorso anno con la terza che era più piccolina questo dettaglio ci ha velocizzato non poco le operazioni di lavaggio😅), è funzionale nella sua estrema semplicità. Non aspettatevi il lusso, ma pulizia, concretezza e praticità. Per il resto, tutto funziona alla perfezione, come un ingranaggio ben oliato;  le macchinine dello staff si vedono costantemente girare per il camping per provvedere ad eventuali interventi/riparazioni; l'isola ecologica è ben organizzata e ben tenuta; non essendo noi "animali sociali" non abbiamo sfruttato l'animazione ma abbiamo molto apprezzato il fatto che  sia presente ma non  invadente; lo staff sempre sorridente e cordiale; tanti piccoli servizi per aiutare gli ospiti a rendere la loro vacanza più possibile perfetta. La ragazza al bar, giovanissima, sempre cordiale e sorridente. Insomma, si vede che, dietro le quinte c'è tanto, tanto lavoro di squadra.  Noi abbiamo optato per la spiagga libera di Pedaso, con acqua bassa e calma e sabbia, perfetta per bambini e mai affollata, ma volendo ci sono dei lidi in convenzione con servizio navetta. Insomma, una settimana di relax immersi nel verde. Non facciamo che consigliare il Garden River ad amici e conoscenti che cerchino un alloggio semplice ad un budget contenuto e che apprezzino la natura.  Per noi che abbiamo un'unica settimana di ferie a disposizione, veramente una coccola che ci rigenera.…</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t xml:space="preserve">Parcheggio gratuito, Con accesso a Internet gratuito, Piscina, Bar/lounge, Noleggio di biciclette, Biciclette disponibili, Area giochi interna per bambini, Attività per bambini/famiglie, Internet, Piscina a sfioro, Piscina per adulti, Piscina all'aperto, Piscina piccola, Piscina recintata, Ristorante, Colazione disponibile, Freccette, Intrattenimento serale, Pesca, Karaoke, Ping pong, Miniclub, Piscina per bambini, Giochi all'aperto per bambini, Seggioloni disponibili, Animali domestici ammessi, Navetta o servizio taxi gratis, Servizio navetta, Hotel per non fumatori, Angolo cottura, Frigorifero, Utensili da cucina, Camere non fumatori, Camere per famiglie, </t>
         </is>
@@ -621,6 +656,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>82 €</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Bar/lounge, Spiaggia, Sala giochi, Parco giochi per bambini, Attività per bambini/famiglie, Parcheggio, Wi-Fi, Piscina all'aperto, Ristorante, Colazione disponibile, Pasti per bambini, Menù dietetici speciali, Escursioni, Campo da tennis, Tour in bicicletta, Intrattenimento serale, Ping pong, Tour a piedi, Parco acquatico esterno alla struttura, Scivolo acquatico, Piscina per bambini, Giochi all'aperto per bambini, Seggioloni disponibili, Animali domestici ammessi, Centro congressi con accesso a Internet, Strutture per conferenze, Sala banchetti, Sale riunioni, Concierge, Hotel per non fumatori, Arredi esterni, Lounge/sala TV in comune, Ombrelloni, Servizio lavanderia, Lavanderia self-service, Aria condizionata, Sala da pranzo, Servizio di pulizia, Balcone privato, Bollitore per tè/caffè, Angolo cottura, TV a schermo piatto, Bidet, Cassaforte, Zona soggiorno, Sala da pranzo separata, Area soggiorno separata, Divano, Armadio/cabina, Appendiabiti, Bagni privati, Pavimento in piastrelle/marmo, Frigorifero, Piano cottura, Bollitore elettrico, Utensili da cucina, Cabina doccia, Bagno/doccia, Asciugacapelli, Vista sulle montagne, Vista sull'oceano, Vista sulla piscina, Camere non fumatori, Suite, Camere per famiglie, </t>
         </is>
       </c>
@@ -646,6 +686,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>140 €</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Animali domestici ammessi, Angolo cottura, </t>
         </is>
       </c>
@@ -671,6 +716,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Caffetteria, Noleggio di biciclette, Aerobica, Servizio di babysitter, Parco giochi per bambini, Wi-Fi, Ristorante, Colazione disponibile, Pasti per bambini, Zona pranzo all'aperto, Freccette, Personale di intrattenimento, Intrattenimento serale, Pesca, Karaoke, Ping pong, Attività per bambini/famiglie, Miniclub, Giochi all'aperto per bambini, Seggioloni disponibili, Animali domestici ammessi, Trasporti per l'aeroporto, Servizio taxi, Trattamenti per il viso, Massaggio completo, Manicure, Massaggio, Servizi di ceretta, Accesso diretto alle piste da sci, Sicurezza 24 ore su 24, Area barbecue, Concierge, Hotel per non fumatori, Lettini/sedie sdraio, Ombrelloni, Cassetta di pronto soccorso, Infermeria, Ombrello, Check-in/check-out express, Servizio lavanderia, Lavanderia self-service, Servizio stireria, Purificatore d'aria, Aria condizionata, Servizio di pulizia, Balcone privato, Bagni privati, Angolo cottura, TV satellitare/via cavo, Bidet, Pavimento in piastrelle/marmo, Frigorifero, Piano cottura, Utensili da cucina, TV a schermo piatto, Cabina doccia, Asciugacapelli, Vista sulla piscina, Camere non fumatori, Camere per famiglie, Camere per fumatori disponibili, </t>
         </is>
       </c>
@@ -696,6 +746,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parcheggio gratuito, Con accesso a Internet gratuito, Bar/lounge, Spiaggia, Noleggio di biciclette, Miniclub, Giochi all'aperto per bambini, Animali domestici ammessi, Parcheggio in strada, Ristorante, Pasti per bambini, Snack bar, Personale di intrattenimento, Intrattenimento serale, Ping pong, Servizio navetta, Area barbecue, Minimarket, Hotel per non fumatori, Servizio lavanderia, Aria condizionata, Spiaggia privata, Zona soggiorno, Acqua in bottiglia, Angolo cottura, Frigorifero, Utensili da cucina, TV a schermo piatto, Camere non fumatori, Camere per famiglie, Camere per fumatori disponibili, </t>
         </is>
       </c>
@@ -719,7 +774,12 @@
           <t>Abbiamo affittato una delle casette. Posto raggiungibile agevolmente da Civitanova Alta seguendo Google Maps. La casa è dotata di tutto il necessario, potrete trovare una cucina funzionante con stoviglie già presenti. C’è l’aria condizionata. All’esterno una piscina rilassante ad uso privato di chi alloggia è un piccolo parco con giochi per bambini. Tutto molto rilassante. C’è il WiFi che funziona perfettamente e anche la possibilità di fare lavatrici se necessario. A noi Vodafone per chiamare non prendeva (forse altri operatori vanno bene) ma comunque si può usare la connessione per chiamare con Whatsapp.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>non disponibile</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -741,6 +801,11 @@
         </is>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>55 €</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t xml:space="preserve">Parcheggio gratuito, Internet ad alta velocità gratuito (WiFi), Piscina, Lezioni di yoga, Bar a bordo piscina, Spiaggia, Noleggio di biciclette, Attività per bambini/famiglie, Parcheggio custodito, Wi-Fi, Teli da piscina/mare, Piscina con vista, Piscina all'aperto, Piscina con estremità bassa, Piscina recintata, Ristorante, Pasti per bambini, Giochi all'aperto per bambini, Animali domestici ammessi, Trasporti per l'aeroporto, Servizio navetta, Sale riunioni, Area barbecue, Deposito bagagli, Hotel per non fumatori, Arredi esterni, Area picnic, Lettini/sedie sdraio, Terrazza solarium, Reception 24 ore su 24, Servizio lavanderia, Acqua in bottiglia, Angolo cottura, Camere per famiglie, </t>
         </is>

</xml_diff>

<commit_message>
inserita colonna id su general dataset tripadvisor. i camping con gli id in comune tengono l'id di booking
</commit_message>
<xml_diff>
--- a/datasets/general_data_dataset_tripadvisor.xlsx
+++ b/datasets/general_data_dataset_tripadvisor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miles\Downloads\progetto_bda-main\datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simo\Desktop\progetto_bda-main\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D35372-4ACE-4704-89B2-511B69AB817C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6F6CDD-267E-400A-8CC8-CD3F765104DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1305" yWindow="915" windowWidth="31755" windowHeight="13755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="165">
   <si>
     <t>name</t>
   </si>
@@ -434,13 +434,94 @@
   </si>
   <si>
     <t>https://www.tripadvisor.com/Hotel_Review-g608900-d1520372-Reviews-Camping_Club_Internazionale-Sirolo_Province_of_Ancona_Marche.html</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Camping-Club-Internazionale-Sirolo</t>
+  </si>
+  <si>
+    <t>La-Risacca-Camping-Village-Formule-Hotel-Porto-Sant-Elpidio</t>
+  </si>
+  <si>
+    <t>Reviews-Girasole-Eco-Family-Village-Marina-Palmense-Fermo</t>
+  </si>
+  <si>
+    <t>Green-Garden-Camping-Village-Sirolo</t>
+  </si>
+  <si>
+    <t>Centro-Vacanze-Garden-River-Altidona</t>
+  </si>
+  <si>
+    <t>Amapolas-Villaggio-Camping-Mombaroccio</t>
+  </si>
+  <si>
+    <t>Villaggio-Turistico-Residence-Mare-Fermo</t>
+  </si>
+  <si>
+    <t>Camping-Villaggio-Cortina-Senigallia</t>
+  </si>
+  <si>
+    <t>La-Mimosa-Camping-Fano</t>
+  </si>
+  <si>
+    <t>Camping-Vettore-Montegallo</t>
+  </si>
+  <si>
+    <t>Camping-Monte-Prata-Castelsantangelo-sul-Nera</t>
+  </si>
+  <si>
+    <t>Camping-Centro-Turistico-Belvedere-Civitanova-Marche</t>
+  </si>
+  <si>
+    <t>Camping-Stella-Maris-Fano</t>
+  </si>
+  <si>
+    <t>Conero-Azzurro-Numana</t>
+  </si>
+  <si>
+    <t>Camping-Don-Diego-Grottammare</t>
+  </si>
+  <si>
+    <t>Camping-Lpre-Ostra</t>
+  </si>
+  <si>
+    <t>Camping-Bellamare-Porto-Recanati</t>
+  </si>
+  <si>
+    <t>Camping-Reno-Sirolo</t>
+  </si>
+  <si>
+    <t>Camping-Summerland-Senigallia</t>
+  </si>
+  <si>
+    <t>Camping-Gabicce-Monte-Gabicce-Monte</t>
+  </si>
+  <si>
+    <t>villaggio-camping-blu</t>
+  </si>
+  <si>
+    <t>Natural-Village-Resort-Porto-Potenza-Picena</t>
+  </si>
+  <si>
+    <t>camping-village-mar-y-sierra</t>
+  </si>
+  <si>
+    <t>glamping-poggio-imperiale-marche-1</t>
+  </si>
+  <si>
+    <t>civettuola</t>
+  </si>
+  <si>
+    <t>camping-paradiso</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -453,6 +534,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -462,7 +551,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -485,17 +574,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -796,7 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
@@ -804,10 +910,11 @@
     <col min="4" max="4" width="20.5703125" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
-    <col min="7" max="7" width="48.85546875" customWidth="1"/>
+    <col min="7" max="7" width="58.28515625" customWidth="1"/>
+    <col min="8" max="8" width="73" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -826,8 +933,11 @@
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -846,11 +956,14 @@
       <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -869,11 +982,14 @@
       <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -892,11 +1008,14 @@
       <c r="F4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -915,11 +1034,14 @@
       <c r="F5" t="s">
         <v>26</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -938,11 +1060,14 @@
       <c r="F6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -961,11 +1086,14 @@
       <c r="F7" t="s">
         <v>36</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -984,11 +1112,14 @@
       <c r="F8" t="s">
         <v>42</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1007,11 +1138,14 @@
       <c r="F9" t="s">
         <v>47</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1030,11 +1164,14 @@
       <c r="F10" t="s">
         <v>52</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1053,11 +1190,14 @@
       <c r="F11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1073,11 +1213,14 @@
       <c r="E12" t="s">
         <v>9</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1096,11 +1239,14 @@
       <c r="F13" t="s">
         <v>66</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="3" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1119,11 +1265,14 @@
       <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="3" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1142,11 +1291,14 @@
       <c r="F15" t="s">
         <v>76</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1165,11 +1317,14 @@
       <c r="F16" t="s">
         <v>81</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1188,11 +1343,14 @@
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1211,11 +1369,14 @@
       <c r="F18" t="s">
         <v>91</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1234,11 +1395,14 @@
       <c r="F19" t="s">
         <v>96</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1257,11 +1421,14 @@
       <c r="F20" t="s">
         <v>101</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1280,11 +1447,14 @@
       <c r="F21" t="s">
         <v>106</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1303,11 +1473,14 @@
       <c r="F22" t="s">
         <v>111</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="3" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1326,11 +1499,14 @@
       <c r="F23" t="s">
         <v>116</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="3" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1349,11 +1525,14 @@
       <c r="F24" t="s">
         <v>121</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="3" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1372,11 +1551,14 @@
       <c r="F25" t="s">
         <v>126</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1395,11 +1577,14 @@
       <c r="F26" t="s">
         <v>131</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="3" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1418,11 +1603,42 @@
       <c r="F27" t="s">
         <v>136</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="3" t="s">
         <v>137</v>
       </c>
+      <c r="H27" t="s">
+        <v>139</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{960FFFA2-0633-459B-BD9F-4613A7083B9E}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{A550377A-ED7F-4FE3-9A08-E88FB202DD51}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{89F969BC-1B33-49C6-83FF-F6DFB5E88FDF}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{8EFDDA4E-481D-4973-9741-459E5AE67D89}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{3723E773-C5EC-459E-8355-BE11A1A7908D}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{2CB56719-C23B-4A39-B82B-82CA434F36F1}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{E2691E92-57F9-400F-990B-AC0DD1436005}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{76F55FA6-2A1C-4403-87E0-CCC7CEA92161}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{138B2497-3E07-4448-8C2B-204D0C003633}"/>
+    <hyperlink ref="G11" r:id="rId10" xr:uid="{728C4F5F-3A49-493A-B5B7-F417E0E17A49}"/>
+    <hyperlink ref="G12" r:id="rId11" xr:uid="{D76AF28A-CE57-47D2-80D2-B789E1F1174C}"/>
+    <hyperlink ref="G13" r:id="rId12" xr:uid="{EA06E08E-EC50-4C58-AD94-1655DF8D48A0}"/>
+    <hyperlink ref="G14" r:id="rId13" xr:uid="{5DE905EF-80BC-446F-A312-9341AB0B50D5}"/>
+    <hyperlink ref="G15" r:id="rId14" xr:uid="{45F6B3AD-125F-4155-8206-11F6CD211115}"/>
+    <hyperlink ref="G17" r:id="rId15" xr:uid="{90D28D3D-6AD0-46A1-AB15-FCD8AC4BD65D}"/>
+    <hyperlink ref="G16" r:id="rId16" xr:uid="{FCA5F3AE-F1CE-41F9-9178-F39E1C7B1448}"/>
+    <hyperlink ref="G18" r:id="rId17" xr:uid="{4613D0F7-8ED4-4C5C-BA38-AE3D1FE48AF3}"/>
+    <hyperlink ref="G19" r:id="rId18" xr:uid="{4F9F2512-E5FE-4029-A500-FCE8AF6DA93A}"/>
+    <hyperlink ref="G20" r:id="rId19" xr:uid="{9CED43EB-AF62-4868-8237-33BF89E84C88}"/>
+    <hyperlink ref="G21" r:id="rId20" xr:uid="{F0EAC6EE-0EDC-4629-B250-75F95B540FB4}"/>
+    <hyperlink ref="G22" r:id="rId21" xr:uid="{D93CE2B5-FBF8-4D98-8CE2-B4DE099AA032}"/>
+    <hyperlink ref="G23" r:id="rId22" xr:uid="{020D1DC9-D2E8-4DAB-83FB-E97ABC1D14FE}"/>
+    <hyperlink ref="G24" r:id="rId23" xr:uid="{E9FF066A-24DA-41D9-91F9-466AF64A6831}"/>
+    <hyperlink ref="G25" r:id="rId24" xr:uid="{473D5A4F-10ED-46B2-BABD-8CD49549B516}"/>
+    <hyperlink ref="G26" r:id="rId25" xr:uid="{FC5A67C9-AB48-4C55-979D-3E7FCCF693A1}"/>
+    <hyperlink ref="G27" r:id="rId26" xr:uid="{1255A9CC-CC9D-47E1-9B9F-A9ABFB8CB22C}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
general data con ID
</commit_message>
<xml_diff>
--- a/datasets/general_data_dataset_tripadvisor.xlsx
+++ b/datasets/general_data_dataset_tripadvisor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Simo\Desktop\progetto_bda-main\datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miles\Downloads\progetto_bda-main\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6F6CDD-267E-400A-8CC8-CD3F765104DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B02C5F11-731E-4610-99FD-77086112D99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="915" windowWidth="31755" windowHeight="13755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -436,92 +436,92 @@
     <t>https://www.tripadvisor.com/Hotel_Review-g608900-d1520372-Reviews-Camping_Club_Internazionale-Sirolo_Province_of_Ancona_Marche.html</t>
   </si>
   <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>Camping-Club-Internazionale-Sirolo</t>
-  </si>
-  <si>
-    <t>La-Risacca-Camping-Village-Formule-Hotel-Porto-Sant-Elpidio</t>
-  </si>
-  <si>
-    <t>Reviews-Girasole-Eco-Family-Village-Marina-Palmense-Fermo</t>
-  </si>
-  <si>
-    <t>Green-Garden-Camping-Village-Sirolo</t>
-  </si>
-  <si>
-    <t>Centro-Vacanze-Garden-River-Altidona</t>
-  </si>
-  <si>
-    <t>Amapolas-Villaggio-Camping-Mombaroccio</t>
-  </si>
-  <si>
-    <t>Villaggio-Turistico-Residence-Mare-Fermo</t>
-  </si>
-  <si>
-    <t>Camping-Villaggio-Cortina-Senigallia</t>
-  </si>
-  <si>
-    <t>La-Mimosa-Camping-Fano</t>
-  </si>
-  <si>
-    <t>Camping-Vettore-Montegallo</t>
-  </si>
-  <si>
-    <t>Camping-Monte-Prata-Castelsantangelo-sul-Nera</t>
-  </si>
-  <si>
-    <t>Camping-Centro-Turistico-Belvedere-Civitanova-Marche</t>
-  </si>
-  <si>
-    <t>Camping-Stella-Maris-Fano</t>
-  </si>
-  <si>
-    <t>Conero-Azzurro-Numana</t>
-  </si>
-  <si>
-    <t>Camping-Don-Diego-Grottammare</t>
-  </si>
-  <si>
-    <t>Camping-Lpre-Ostra</t>
-  </si>
-  <si>
-    <t>Camping-Bellamare-Porto-Recanati</t>
-  </si>
-  <si>
-    <t>Camping-Reno-Sirolo</t>
-  </si>
-  <si>
-    <t>Camping-Summerland-Senigallia</t>
-  </si>
-  <si>
-    <t>Camping-Gabicce-Monte-Gabicce-Monte</t>
-  </si>
-  <si>
-    <t>villaggio-camping-blu</t>
-  </si>
-  <si>
-    <t>Natural-Village-Resort-Porto-Potenza-Picena</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>natural-village-resort</t>
+  </si>
+  <si>
+    <t>casale-civetta</t>
+  </si>
+  <si>
+    <t>conero-azzurro</t>
+  </si>
+  <si>
+    <t>green-garden-camping-village</t>
+  </si>
+  <si>
+    <t>amapolas-villaggio-&amp;-camping</t>
+  </si>
+  <si>
+    <t>camping-villaggio-cortina</t>
+  </si>
+  <si>
+    <t>camping-vettore</t>
+  </si>
+  <si>
+    <t>camping-gabicce-monte</t>
+  </si>
+  <si>
+    <t>la-mimosa-camping</t>
+  </si>
+  <si>
+    <t>camping-lpre</t>
+  </si>
+  <si>
+    <t>camping-don-diego</t>
+  </si>
+  <si>
+    <t>camping-monte-prata</t>
+  </si>
+  <si>
+    <t>camping-paradiso</t>
+  </si>
+  <si>
+    <t>camping-centro-turistico-belvedere</t>
+  </si>
+  <si>
+    <t>camping-bellamare</t>
+  </si>
+  <si>
+    <t>la-risacca-camping-village</t>
+  </si>
+  <si>
+    <t>centro-vacanze-garden-river</t>
+  </si>
+  <si>
+    <t>residence-mare</t>
+  </si>
+  <si>
+    <t>camping-reno</t>
+  </si>
+  <si>
+    <t>girasole-eco-family-village</t>
+  </si>
+  <si>
+    <t>camping-blu-fantasy</t>
   </si>
   <si>
     <t>camping-village-mar-y-sierra</t>
   </si>
   <si>
-    <t>glamping-poggio-imperiale-marche-1</t>
-  </si>
-  <si>
-    <t>civettuola</t>
-  </si>
-  <si>
-    <t>camping-paradiso</t>
+    <t>camping-stella-maris</t>
+  </si>
+  <si>
+    <t>camping-summerland</t>
+  </si>
+  <si>
+    <t>poggio-imperiale-marche</t>
+  </si>
+  <si>
+    <t>camping-club-internazionale</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -533,14 +533,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -586,11 +578,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -598,10 +589,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -905,13 +894,13 @@
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
     <col min="4" max="4" width="20.5703125" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
-    <col min="7" max="7" width="58.28515625" customWidth="1"/>
-    <col min="8" max="8" width="73" customWidth="1"/>
+    <col min="7" max="7" width="46" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -956,11 +945,11 @@
       <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -982,11 +971,11 @@
       <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" t="s">
         <v>16</v>
       </c>
       <c r="H3" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1008,11 +997,11 @@
       <c r="F4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" t="s">
         <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1034,7 +1023,7 @@
       <c r="F5" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" t="s">
         <v>27</v>
       </c>
       <c r="H5" t="s">
@@ -1060,7 +1049,7 @@
       <c r="F6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" t="s">
         <v>32</v>
       </c>
       <c r="H6" t="s">
@@ -1086,11 +1075,11 @@
       <c r="F7" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" t="s">
         <v>37</v>
       </c>
       <c r="H7" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1112,11 +1101,11 @@
       <c r="F8" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" t="s">
         <v>43</v>
       </c>
       <c r="H8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1138,11 +1127,11 @@
       <c r="F9" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" t="s">
         <v>48</v>
       </c>
       <c r="H9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1164,11 +1153,11 @@
       <c r="F10" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" t="s">
         <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1190,11 +1179,11 @@
       <c r="F11" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" t="s">
         <v>58</v>
       </c>
       <c r="H11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1213,11 +1202,11 @@
       <c r="E12" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" t="s">
         <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1239,11 +1228,11 @@
       <c r="F13" t="s">
         <v>66</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" t="s">
         <v>67</v>
       </c>
       <c r="H13" t="s">
-        <v>163</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1265,7 +1254,7 @@
       <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" t="s">
         <v>72</v>
       </c>
       <c r="H14" t="s">
@@ -1291,11 +1280,11 @@
       <c r="F15" t="s">
         <v>76</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" t="s">
         <v>77</v>
       </c>
       <c r="H15" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1317,11 +1306,11 @@
       <c r="F16" t="s">
         <v>81</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" t="s">
         <v>82</v>
       </c>
       <c r="H16" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1343,11 +1332,11 @@
       <c r="F17" t="s">
         <v>86</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" t="s">
         <v>87</v>
       </c>
       <c r="H17" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1369,11 +1358,11 @@
       <c r="F18" t="s">
         <v>91</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" t="s">
         <v>92</v>
       </c>
       <c r="H18" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1395,11 +1384,11 @@
       <c r="F19" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" t="s">
         <v>97</v>
       </c>
       <c r="H19" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1421,11 +1410,11 @@
       <c r="F20" t="s">
         <v>101</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" t="s">
         <v>102</v>
       </c>
       <c r="H20" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1447,11 +1436,11 @@
       <c r="F21" t="s">
         <v>106</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" t="s">
         <v>107</v>
       </c>
       <c r="H21" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1473,11 +1462,11 @@
       <c r="F22" t="s">
         <v>111</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" t="s">
         <v>112</v>
       </c>
       <c r="H22" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1499,11 +1488,11 @@
       <c r="F23" t="s">
         <v>116</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" t="s">
         <v>117</v>
       </c>
       <c r="H23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1525,11 +1514,11 @@
       <c r="F24" t="s">
         <v>121</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" t="s">
         <v>122</v>
       </c>
       <c r="H24" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1551,11 +1540,11 @@
       <c r="F25" t="s">
         <v>126</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" t="s">
         <v>127</v>
       </c>
       <c r="H25" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1577,11 +1566,11 @@
       <c r="F26" t="s">
         <v>131</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" t="s">
         <v>132</v>
       </c>
       <c r="H26" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1603,42 +1592,15 @@
       <c r="F27" t="s">
         <v>136</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" t="s">
         <v>137</v>
       </c>
       <c r="H27" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{960FFFA2-0633-459B-BD9F-4613A7083B9E}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{A550377A-ED7F-4FE3-9A08-E88FB202DD51}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{89F969BC-1B33-49C6-83FF-F6DFB5E88FDF}"/>
-    <hyperlink ref="G5" r:id="rId4" xr:uid="{8EFDDA4E-481D-4973-9741-459E5AE67D89}"/>
-    <hyperlink ref="G6" r:id="rId5" xr:uid="{3723E773-C5EC-459E-8355-BE11A1A7908D}"/>
-    <hyperlink ref="G7" r:id="rId6" xr:uid="{2CB56719-C23B-4A39-B82B-82CA434F36F1}"/>
-    <hyperlink ref="G8" r:id="rId7" xr:uid="{E2691E92-57F9-400F-990B-AC0DD1436005}"/>
-    <hyperlink ref="G9" r:id="rId8" xr:uid="{76F55FA6-2A1C-4403-87E0-CCC7CEA92161}"/>
-    <hyperlink ref="G10" r:id="rId9" xr:uid="{138B2497-3E07-4448-8C2B-204D0C003633}"/>
-    <hyperlink ref="G11" r:id="rId10" xr:uid="{728C4F5F-3A49-493A-B5B7-F417E0E17A49}"/>
-    <hyperlink ref="G12" r:id="rId11" xr:uid="{D76AF28A-CE57-47D2-80D2-B789E1F1174C}"/>
-    <hyperlink ref="G13" r:id="rId12" xr:uid="{EA06E08E-EC50-4C58-AD94-1655DF8D48A0}"/>
-    <hyperlink ref="G14" r:id="rId13" xr:uid="{5DE905EF-80BC-446F-A312-9341AB0B50D5}"/>
-    <hyperlink ref="G15" r:id="rId14" xr:uid="{45F6B3AD-125F-4155-8206-11F6CD211115}"/>
-    <hyperlink ref="G17" r:id="rId15" xr:uid="{90D28D3D-6AD0-46A1-AB15-FCD8AC4BD65D}"/>
-    <hyperlink ref="G16" r:id="rId16" xr:uid="{FCA5F3AE-F1CE-41F9-9178-F39E1C7B1448}"/>
-    <hyperlink ref="G18" r:id="rId17" xr:uid="{4613D0F7-8ED4-4C5C-BA38-AE3D1FE48AF3}"/>
-    <hyperlink ref="G19" r:id="rId18" xr:uid="{4F9F2512-E5FE-4029-A500-FCE8AF6DA93A}"/>
-    <hyperlink ref="G20" r:id="rId19" xr:uid="{9CED43EB-AF62-4868-8237-33BF89E84C88}"/>
-    <hyperlink ref="G21" r:id="rId20" xr:uid="{F0EAC6EE-0EDC-4629-B250-75F95B540FB4}"/>
-    <hyperlink ref="G22" r:id="rId21" xr:uid="{D93CE2B5-FBF8-4D98-8CE2-B4DE099AA032}"/>
-    <hyperlink ref="G23" r:id="rId22" xr:uid="{020D1DC9-D2E8-4DAB-83FB-E97ABC1D14FE}"/>
-    <hyperlink ref="G24" r:id="rId23" xr:uid="{E9FF066A-24DA-41D9-91F9-466AF64A6831}"/>
-    <hyperlink ref="G25" r:id="rId24" xr:uid="{473D5A4F-10ED-46B2-BABD-8CD49549B516}"/>
-    <hyperlink ref="G26" r:id="rId25" xr:uid="{FC5A67C9-AB48-4C55-979D-3E7FCCF693A1}"/>
-    <hyperlink ref="G27" r:id="rId26" xr:uid="{1255A9CC-CC9D-47E1-9B9F-A9ABFB8CB22C}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>